<commit_message>
Add JS Format formula column to Excel for easy copy-paste into faq-data.js
</commit_message>
<xml_diff>
--- a/faq-sample.xlsx
+++ b/faq-sample.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +60,13 @@
       <color rgb="002B4DB3"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Courier New"/>
+      <color rgb="001C2D6E"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +98,11 @@
         <fgColor rgb="00FFF1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002B4DB3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -120,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +197,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,13 +569,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -583,6 +600,11 @@
           <t>answer</t>
         </is>
       </c>
+      <c r="E1" s="23" t="inlineStr">
+        <is>
+          <t>JS Format (copy this → paste into faq-data.js)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="52" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -603,6 +625,10 @@
           <t>Yes, you can try us for free for 30 days. If you want, we'll provide you with a free 30-minute onboarding call to get you up and running as quickly as possible.</t>
         </is>
       </c>
+      <c r="E2" s="24">
+        <f>"  { id:"&amp;A2&amp;", category:\""&amp;B2&amp;"\", question:\""&amp;C2&amp;"\", answer:\""&amp;D2&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="5" t="n">
@@ -623,6 +649,10 @@
           <t>Of course! Our pricing scales with your company. Chat to our friendly team to find a solution that works for you as you grow. You can upgrade or downgrade at any time from your account settings.</t>
         </is>
       </c>
+      <c r="E3" s="24">
+        <f>"  { id:"&amp;A3&amp;", category:\""&amp;B3&amp;"\", question:\""&amp;C3&amp;"\", answer:\""&amp;D3&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="52" customHeight="1">
       <c r="A4" s="8" t="n">
@@ -643,6 +673,10 @@
           <t>We understand that things change. You can cancel your plan at any time and we'll refund you the difference already paid. No questions asked — we want you to be happy with your choice.</t>
         </is>
       </c>
+      <c r="E4" s="24">
+        <f>"  { id:"&amp;A4&amp;", category:\""&amp;B4&amp;"\", question:\""&amp;C4&amp;"\", answer:\""&amp;D4&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="8" t="n">
@@ -663,6 +697,10 @@
           <t>At the moment, the only way to add additional information to invoices is to add the information to the workspace's name manually. We're working on a full invoice customisation feature — stay tuned!</t>
         </is>
       </c>
+      <c r="E5" s="24">
+        <f>"  { id:"&amp;A5&amp;", category:\""&amp;B5&amp;"\", question:\""&amp;C5&amp;"\", answer:\""&amp;D5&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -683,6 +721,10 @@
           <t>Once you have purchased the UI kit, you will have access to all of the future updates, free of charge. We'll let you know about releases via email and in-app notifications. There is no annual renewal fee.</t>
         </is>
       </c>
+      <c r="E6" s="24">
+        <f>"  { id:"&amp;A6&amp;", category:\""&amp;B6&amp;"\", question:\""&amp;C6&amp;"\", answer:\""&amp;D6&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -703,6 +745,10 @@
           <t>Just a one-time payment! No recurring charges or surprises, we promise. We're just as sick of recurring charges as you are. Pay once, use forever.</t>
         </is>
       </c>
+      <c r="E7" s="24">
+        <f>"  { id:"&amp;A7&amp;", category:\""&amp;B7&amp;"\", question:\""&amp;C7&amp;"\", answer:\""&amp;D7&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="11" t="n">
@@ -723,6 +769,10 @@
           <t>You can reset your password from the login screen by clicking "Forgot password". We'll send a reset link to your registered email address. The link expires after 24 hours for security. If you don't receive the email, check your spam folder.</t>
         </is>
       </c>
+      <c r="E8" s="24">
+        <f>"  { id:"&amp;A8&amp;", category:\""&amp;B8&amp;"\", question:\""&amp;C8&amp;"\", answer:\""&amp;D8&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="A9" s="11" t="n">
@@ -743,6 +793,10 @@
           <t>Yes! Our Team and Enterprise plans support multiple seats. Each user gets their own login credentials and personalised settings. Admins can manage permissions, add or remove members, and view usage across all seats from the dashboard.</t>
         </is>
       </c>
+      <c r="E9" s="24">
+        <f>"  { id:"&amp;A9&amp;", category:\""&amp;B9&amp;"\", question:\""&amp;C9&amp;"\", answer:\""&amp;D9&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="52" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -763,6 +817,10 @@
           <t>The Enterprise plan includes everything in Team, plus: SSO/SAML authentication, dedicated account manager, custom SLAs, audit logs, advanced role-based access control, and priority 24/7 support. Contact us for custom pricing.</t>
         </is>
       </c>
+      <c r="E10" s="24">
+        <f>"  { id:"&amp;A10&amp;", category:\""&amp;B10&amp;"\", question:\""&amp;C10&amp;"\", answer:\""&amp;D10&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="52" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -783,6 +841,10 @@
           <t>Absolutely. We offer a 50% discount for verified non-profit organisations and educational institutions. Simply contact our support team with proof of your status and we'll apply the discount to your account within one business day.</t>
         </is>
       </c>
+      <c r="E11" s="24">
+        <f>"  { id:"&amp;A11&amp;", category:\""&amp;B11&amp;"\", question:\""&amp;C11&amp;"\", answer:\""&amp;D11&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="52" customHeight="1">
       <c r="A12" s="11" t="n">
@@ -803,6 +865,10 @@
           <t>You can request account deletion from Settings → Account → Delete Account. Your data will be permanently removed within 30 days in accordance with our data retention policy. This action is irreversible, so please export any data you need beforehand.</t>
         </is>
       </c>
+      <c r="E12" s="24">
+        <f>"  { id:"&amp;A12&amp;", category:\""&amp;B12&amp;"\", question:\""&amp;C12&amp;"\", answer:\""&amp;D12&amp;"\" },"</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="52" customHeight="1">
       <c r="A13" s="8" t="n">
@@ -822,6 +888,10 @@
         <is>
           <t>We accept all major credit and debit cards (Visa, Mastercard, Amex, Discover), PayPal, and bank transfers for annual Enterprise contracts. All payments are processed securely via Stripe. We do not store card details on our servers.</t>
         </is>
+      </c>
+      <c r="E13" s="24">
+        <f>"  { id:"&amp;A13&amp;", category:\""&amp;B13&amp;"\", question:\""&amp;C13&amp;"\", answer:\""&amp;D13&amp;"\" },"</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>